<commit_message>
Fixed names and links. Also fixed the decimal saving in Excel
</commit_message>
<xml_diff>
--- a/Manual calc.xlsx
+++ b/Manual calc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6d20085048815992/Documenti/GitHub/ranking_aus_super/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="467" documentId="8_{6B50DBFC-E840-4F93-9C07-3F647D2188CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79CA765E-30C6-41DF-B90F-D062F60B2017}"/>
+  <xr:revisionPtr revIDLastSave="469" documentId="8_{6B50DBFC-E840-4F93-9C07-3F647D2188CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{821A9710-D872-4832-8638-DDDFBA467699}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{463C025B-1AEA-4D48-A61E-6EBBD6EBE81E}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{463C025B-1AEA-4D48-A61E-6EBBD6EBE81E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="2" r:id="rId1"/>
@@ -180,9 +180,6 @@
     <t>HOSTPLUS_fees-and-costs-guide.pdf.coredownload.pdf</t>
   </si>
   <si>
-    <t>https://hostplus.com.au/about-us/legals/pds#accordion-f7de90f571-item-cd98b24680</t>
-  </si>
-  <si>
     <t>IOOF MYSUPER</t>
   </si>
   <si>
@@ -331,6 +328,9 @@
   </si>
   <si>
     <t>Active Super Saver</t>
+  </si>
+  <si>
+    <t>https://www.hesta.com.au/members/your-superannuation/fees-and-costs</t>
   </si>
 </sst>
 </file>
@@ -883,10 +883,7 @@
         <v>43</v>
       </c>
       <c r="B13" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" t="s">
-        <v>45</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -896,168 +893,171 @@
       <c r="B14" t="s">
         <v>45</v>
       </c>
+      <c r="C14" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" t="s">
         <v>47</v>
-      </c>
-      <c r="B15" t="s">
-        <v>49</v>
-      </c>
-      <c r="C15" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C18" t="s">
         <v>58</v>
-      </c>
-      <c r="B18" t="s">
-        <v>57</v>
-      </c>
-      <c r="C18" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" t="s">
         <v>67</v>
-      </c>
-      <c r="B22" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" t="s">
+        <v>70</v>
+      </c>
+      <c r="C23" t="s">
         <v>69</v>
-      </c>
-      <c r="B23" t="s">
-        <v>71</v>
-      </c>
-      <c r="C23" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" t="s">
         <v>72</v>
-      </c>
-      <c r="B24" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" t="s">
         <v>74</v>
-      </c>
-      <c r="B25" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B27" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" t="s">
         <v>80</v>
-      </c>
-      <c r="C27" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" t="s">
         <v>83</v>
-      </c>
-      <c r="B28" t="s">
-        <v>85</v>
-      </c>
-      <c r="C28" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
+        <v>85</v>
+      </c>
+      <c r="B29" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" t="s">
         <v>86</v>
-      </c>
-      <c r="B29" t="s">
-        <v>90</v>
-      </c>
-      <c r="C29" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
+        <v>92</v>
+      </c>
+      <c r="B31" t="s">
         <v>93</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>94</v>
-      </c>
-      <c r="C31" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1138,55 +1138,55 @@
         <v>44</v>
       </c>
       <c r="O4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="P4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Q4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="R4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="S4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="T4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="U4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="V4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="W4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="X4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Z4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AA4" t="s">
+        <v>81</v>
+      </c>
+      <c r="AB4" t="s">
         <v>82</v>
       </c>
-      <c r="AB4" t="s">
-        <v>83</v>
-      </c>
       <c r="AC4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="AD4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="AE4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:43" x14ac:dyDescent="0.35">
@@ -1337,99 +1337,99 @@
         <v>1.7333333333333334E-4</v>
       </c>
       <c r="H6" s="2">
-        <f>H5/$B$2</f>
+        <f t="shared" ref="H6:O6" si="1">H5/$B$2</f>
         <v>0</v>
       </c>
       <c r="I6" s="2">
-        <f>I5/$B$2</f>
+        <f t="shared" si="1"/>
         <v>4.5066666666666665E-4</v>
       </c>
       <c r="J6" s="2">
-        <f>J5/$B$2</f>
+        <f t="shared" si="1"/>
         <v>1.3333333333333334E-4</v>
       </c>
       <c r="K6" s="2">
-        <f>K5/$B$2</f>
+        <f t="shared" si="1"/>
         <v>4.5066666666666665E-4</v>
       </c>
       <c r="L6" s="2">
-        <f>L5/$B$2</f>
+        <f t="shared" si="1"/>
         <v>5.7200000000000003E-4</v>
       </c>
       <c r="M6" s="2">
-        <f>M5/$B$2</f>
+        <f t="shared" si="1"/>
         <v>3.4666666666666667E-4</v>
       </c>
       <c r="N6" s="2">
-        <f>N5/$B$2</f>
-        <v>5.1999999999999995E-4</v>
-      </c>
-      <c r="O6" s="2">
-        <f>O5/$B$2</f>
-        <v>5.1999999999999995E-4</v>
-      </c>
-      <c r="P6" s="2">
-        <f t="shared" ref="P6:X6" si="1">P5/$B$2</f>
-        <v>3.4319999999999999E-4</v>
-      </c>
-      <c r="Q6" s="2">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R6" s="2">
         <f t="shared" si="1"/>
         <v>5.1999999999999995E-4</v>
       </c>
+      <c r="O6" s="2">
+        <f t="shared" si="1"/>
+        <v>5.1999999999999995E-4</v>
+      </c>
+      <c r="P6" s="2">
+        <f t="shared" ref="P6:W6" si="2">P5/$B$2</f>
+        <v>3.4319999999999999E-4</v>
+      </c>
+      <c r="Q6" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R6" s="2">
+        <f t="shared" si="2"/>
+        <v>5.1999999999999995E-4</v>
+      </c>
       <c r="S6" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.8533333333333333E-4</v>
       </c>
       <c r="T6" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.3333333333333331E-4</v>
       </c>
       <c r="U6" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.9866666666666664E-4</v>
       </c>
       <c r="V6" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.4666666666666667E-4</v>
       </c>
       <c r="W6" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="X6" s="2">
-        <f>X5/$B$2</f>
+        <f t="shared" ref="X6:AE6" si="3">X5/$B$2</f>
         <v>5.1999999999999995E-4</v>
       </c>
       <c r="Y6" s="2">
-        <f>Y5/$B$2</f>
+        <f t="shared" si="3"/>
         <v>2.5999999999999998E-4</v>
       </c>
       <c r="Z6" s="2">
-        <f>Z5/$B$2</f>
+        <f t="shared" si="3"/>
         <v>3.4666666666666667E-4</v>
       </c>
       <c r="AA6" s="2">
-        <f>AA5/$B$2</f>
+        <f t="shared" si="3"/>
         <v>4.0000000000000002E-4</v>
       </c>
       <c r="AB6" s="2">
-        <f>AB5/$B$2</f>
+        <f t="shared" si="3"/>
         <v>6.4000000000000005E-4</v>
       </c>
       <c r="AC6" s="2">
-        <f>AC5/$B$2</f>
+        <f t="shared" si="3"/>
         <v>3.4666666666666667E-4</v>
       </c>
       <c r="AD6" s="2">
-        <f>AD5/$B$2</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AE6" s="2">
-        <f>AE5/$B$2</f>
+        <f t="shared" si="3"/>
         <v>4.4026666666666672E-4</v>
       </c>
       <c r="AF6" s="2"/>
@@ -1557,123 +1557,123 @@
         <v>1</v>
       </c>
       <c r="B8" s="4">
-        <f t="shared" ref="B8:G8" si="2">B6+B7</f>
+        <f t="shared" ref="B8:G8" si="4">B6+B7</f>
         <v>9.8133333333333319E-4</v>
       </c>
       <c r="C8" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.3466666666666666E-3</v>
       </c>
       <c r="D8" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8.0000000000000004E-4</v>
       </c>
       <c r="E8" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>8.0000000000000004E-4</v>
       </c>
       <c r="F8" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.9466666666666669E-3</v>
       </c>
       <c r="G8" s="4">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.5733333333333333E-3</v>
       </c>
       <c r="H8" s="4">
-        <f>H6+H7</f>
+        <f t="shared" ref="H8:O8" si="5">H6+H7</f>
         <v>1.8E-3</v>
       </c>
       <c r="I8" s="4">
-        <f>I6+I7</f>
+        <f t="shared" si="5"/>
         <v>1.9506666666666667E-3</v>
       </c>
       <c r="J8" s="4">
-        <f>J6+J7</f>
+        <f t="shared" si="5"/>
         <v>3.6333333333333335E-3</v>
       </c>
       <c r="K8" s="4">
-        <f>K6+K7</f>
+        <f t="shared" si="5"/>
         <v>2.0506666666666668E-3</v>
       </c>
       <c r="L8" s="4">
-        <f>L6+L7</f>
+        <f t="shared" si="5"/>
         <v>2.372E-3</v>
       </c>
       <c r="M8" s="4">
-        <f>M6+M7</f>
+        <f t="shared" si="5"/>
         <v>1.8466666666666666E-3</v>
       </c>
       <c r="N8" s="4">
-        <f>N6+N7</f>
+        <f t="shared" si="5"/>
         <v>5.1999999999999995E-4</v>
       </c>
       <c r="O8" s="4">
-        <f>O6+O7</f>
+        <f t="shared" si="5"/>
         <v>3.0200000000000001E-3</v>
       </c>
       <c r="P8" s="4">
-        <f t="shared" ref="P8:W8" si="3">P6+P7</f>
+        <f t="shared" ref="P8:W8" si="6">P6+P7</f>
         <v>3.2431999999999999E-3</v>
       </c>
       <c r="Q8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.8E-3</v>
       </c>
       <c r="R8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.4199999999999998E-3</v>
       </c>
       <c r="S8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.7603333333333334E-3</v>
       </c>
       <c r="T8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.1333333333333334E-3</v>
       </c>
       <c r="U8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>1.5986666666666666E-3</v>
       </c>
       <c r="V8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.8466666666666666E-3</v>
       </c>
       <c r="W8" s="4">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>2.5000000000000001E-3</v>
       </c>
       <c r="X8" s="4">
-        <f>X6+X7</f>
+        <f t="shared" ref="X8:AE8" si="7">X6+X7</f>
         <v>1.5200000000000001E-3</v>
       </c>
       <c r="Y8" s="4">
-        <f>Y6+Y7</f>
+        <f t="shared" si="7"/>
         <v>1.8600000000000001E-3</v>
       </c>
       <c r="Z8" s="4">
-        <f>Z6+Z7</f>
+        <f t="shared" si="7"/>
         <v>2.2466666666666668E-3</v>
       </c>
       <c r="AA8" s="4">
-        <f>AA6+AA7</f>
+        <f t="shared" si="7"/>
         <v>2.3E-3</v>
       </c>
       <c r="AB8" s="4">
-        <f>AB6+AB7</f>
+        <f t="shared" si="7"/>
         <v>6.4000000000000005E-4</v>
       </c>
       <c r="AC8" s="4">
-        <f>AC6+AC7</f>
+        <f t="shared" si="7"/>
         <v>2.2466666666666668E-3</v>
       </c>
       <c r="AD8" s="4">
-        <f>AD6+AD7</f>
+        <f t="shared" si="7"/>
         <v>3.3E-3</v>
       </c>
       <c r="AE8" s="4">
-        <f>AE6+AE7</f>
+        <f t="shared" si="7"/>
         <v>1.8402666666666667E-3</v>
       </c>
       <c r="AF8" s="4"/>
@@ -1908,123 +1908,123 @@
         <v>4</v>
       </c>
       <c r="B13" s="5">
-        <f t="shared" ref="B13:G13" si="4">B8+B10+B11</f>
+        <f t="shared" ref="B13:G13" si="8">B8+B10+B11</f>
         <v>5.3813333333333335E-3</v>
       </c>
       <c r="C13" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>7.2466666666666669E-3</v>
       </c>
       <c r="D13" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>1.0600000000000002E-2</v>
       </c>
       <c r="E13" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>6.8000000000000005E-3</v>
       </c>
       <c r="F13" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>7.1466666666666675E-3</v>
       </c>
       <c r="G13" s="5">
-        <f t="shared" si="4"/>
+        <f t="shared" si="8"/>
         <v>6.5733333333333338E-3</v>
       </c>
       <c r="H13" s="5">
-        <f>H8+H10+H11</f>
+        <f t="shared" ref="H13:AE13" si="9">H8+H10+H11</f>
         <v>1.1599999999999999E-2</v>
       </c>
       <c r="I13" s="5">
-        <f>I8+I10+I11</f>
+        <f t="shared" si="9"/>
         <v>7.4506666666666662E-3</v>
       </c>
       <c r="J13" s="5">
-        <f>J8+J10+J11</f>
+        <f t="shared" si="9"/>
         <v>6.7333333333333334E-3</v>
       </c>
       <c r="K13" s="5">
-        <f>K8+K10+K11</f>
+        <f t="shared" si="9"/>
         <v>7.0306666666666668E-3</v>
       </c>
       <c r="L13" s="5">
-        <f>L8+L10+L11</f>
+        <f t="shared" si="9"/>
         <v>7.4720000000000003E-3</v>
       </c>
       <c r="M13" s="5">
-        <f>M8+M10+M11</f>
+        <f t="shared" si="9"/>
         <v>7.0466666666666664E-3</v>
       </c>
       <c r="N13" s="5">
-        <f>N8+N10+N11</f>
+        <f t="shared" si="9"/>
         <v>9.6200000000000001E-3</v>
       </c>
       <c r="O13" s="5">
-        <f>O8+O10+O11</f>
+        <f t="shared" si="9"/>
         <v>9.92E-3</v>
       </c>
       <c r="P13" s="5">
-        <f>P8+P10+P11</f>
+        <f t="shared" si="9"/>
         <v>9.3431999999999994E-3</v>
       </c>
       <c r="Q13" s="5">
-        <f>Q8+Q10+Q11</f>
+        <f t="shared" si="9"/>
         <v>9.4000000000000004E-3</v>
       </c>
       <c r="R13" s="5">
-        <f>R8+R10+R11</f>
+        <f t="shared" si="9"/>
         <v>6.5200000000000006E-3</v>
       </c>
       <c r="S13" s="5">
-        <f>S8+S10+S11</f>
+        <f t="shared" si="9"/>
         <v>7.7603333333333335E-3</v>
       </c>
       <c r="T13" s="5">
-        <f>T8+T10+T11</f>
+        <f t="shared" si="9"/>
         <v>1.2233333333333334E-2</v>
       </c>
       <c r="U13" s="5">
-        <f>U8+U10+U11</f>
+        <f t="shared" si="9"/>
         <v>1.0398666666666667E-2</v>
       </c>
       <c r="V13" s="5">
-        <f>V8+V10+V11</f>
+        <f t="shared" si="9"/>
         <v>7.7466666666666673E-3</v>
       </c>
       <c r="W13" s="5">
-        <f>W8+W10+W11</f>
+        <f t="shared" si="9"/>
         <v>1.0500000000000001E-2</v>
       </c>
       <c r="X13" s="5">
-        <f>X8+X10+X11</f>
+        <f t="shared" si="9"/>
         <v>6.4199999999999995E-3</v>
       </c>
       <c r="Y13" s="5">
-        <f>Y8+Y10+Y11</f>
+        <f t="shared" si="9"/>
         <v>6.4599999999999996E-3</v>
       </c>
       <c r="Z13" s="5">
-        <f>Z8+Z10+Z11</f>
+        <f t="shared" si="9"/>
         <v>8.8466666666666659E-3</v>
       </c>
       <c r="AA13" s="5">
-        <f>AA8+AA10+AA11</f>
+        <f t="shared" si="9"/>
         <v>8.8999999999999999E-3</v>
       </c>
       <c r="AB13" s="5">
-        <f>AB8+AB10+AB11</f>
+        <f t="shared" si="9"/>
         <v>5.1399999999999996E-3</v>
       </c>
       <c r="AC13" s="5">
-        <f>AC8+AC10+AC11</f>
+        <f t="shared" si="9"/>
         <v>7.2466666666666669E-3</v>
       </c>
       <c r="AD13" s="5">
-        <f>AD8+AD10+AD11</f>
+        <f t="shared" si="9"/>
         <v>5.5999999999999999E-3</v>
       </c>
       <c r="AE13" s="5">
-        <f>AE8+AE10+AE11</f>
+        <f t="shared" si="9"/>
         <v>7.8402666666666666E-3</v>
       </c>
       <c r="AF13" s="5"/>
@@ -2042,28 +2042,28 @@
     </row>
     <row r="14" spans="1:43" x14ac:dyDescent="0.35">
       <c r="P14" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="Q14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="U14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="V14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="Z14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="AC14" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AD14" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="AE14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:43" x14ac:dyDescent="0.35">
@@ -2074,7 +2074,7 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E15" t="s">
         <v>25</v>

</xml_diff>